<commit_message>
[문서] MiniVillagerWoman 영어 대사 추가
</commit_message>
<xml_diff>
--- a/Sheets/DialogueData.xlsx
+++ b/Sheets/DialogueData.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tfdkg\UnityProject\Farm\Sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A224F5-17F7-43A5-9954-BB222F561CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1526363D-387C-45C4-BC07-46537F42E3C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{62B5C00F-698F-4EE8-88B3-1AC2C87E7411}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{62B5C00F-698F-4EE8-88B3-1AC2C87E7411}"/>
   </bookViews>
   <sheets>
-    <sheet name="MiniVillagerWoman" sheetId="6" r:id="rId1"/>
+    <sheet name="MiniVillagerWoman_ko" sheetId="6" r:id="rId1"/>
+    <sheet name="MiniVillagerWoman_en" sheetId="7" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MiniVillagerWoman!$D$6:$D$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">MiniVillagerWoman_en!$D$6:$D$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MiniVillagerWoman_ko!$D$6:$D$149</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="66">
   <si>
     <t>$DialogueId$</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1157,6 +1159,225 @@
   </si>
   <si>
     <t>$p 61#역시 그렇지?| 그렇게 생각해?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>$$DialogueData_MiniVillagerWoman_en$$</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>I wonder what would happen if I spent all night in the graveyard?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">#$q 17/18 Sun_old#@, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>what do you think happens to us after we die?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>#$r 17 0 Sun_17#</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>I have no idea.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>#$r 18 40 Sun_18#</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>We come back as spooky ghosts.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>#$r 17 0 Sun_17#We go to Heaven.#$r 18 0 Sun_17#</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>Our energy bodies enter the astral plane</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.#$r 17 30 Sun_nothing#</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>Nothing. We just cease to exist.</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>$p 17#</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>I guess you think nothing would happen, right?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>|</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>Maybe a wicked ghost would appear!</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hmm, interesting…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Well that's an interesting theory!</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>You know, that wouldn't be so bad.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Oh, hi</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Oh, hi @. Taking a break from your work?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ugh... I'm not in a good mood right now.#$e#I said I'm not in a good mood... what do you want?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hey. Sorry in advance if I say anything rude. I didn't get much sleep last night.#$e#What do you want?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>What should I make to eat today…</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Wow, I just realized it's Friday.#$e#Sometimes I completely lose track of time.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The fresh mountain breeze feels so good on days like this.#$e#I wonder if we'll see frogs soon.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>I was planning to catch up on some postponed housework today. #$e#See ya.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>My pet guinea pig David absolutely hates this hot weather. He's quite picky.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The air gets all sticky with honey and fruit juice all summer long. It's dizzying.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Yesterday I was imagining what would happen if Megalodon fought T-Rex.#$q 61/62 spring_6old#@ What do you think? #$r 61 0 spring_61#Megalodon!#$r 62 0 spring_62#T-Rex!#$r 62 0 spring_62#They'd be evenly matched.#$r 61 0 spring_62#No idea.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>$p 61#Yeah, that's right?| You think so?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>I think so too.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hmm, really?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>$y '@, What do you think... Should we judge people by their actions or their intentions?_Actions_Hmm... but everyone has made mistakes before, right?_Intentions_Hmm... but what about when intentions cause harm despite good intentions?_Both_Yeah... we don't have to pick just one. It can depend on the situation too.'#$b#I was just curious what you think...</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1278,7 +1499,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1321,6 +1542,12 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1340,6 +1567,10 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Button" lockText="1"/>
+</file>
+
+<file path=xl/ctrlProps/ctrlProp2.xml><?xml version="1.0" encoding="utf-8"?>
 <formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Button" lockText="1"/>
 </file>
 
@@ -1369,6 +1600,80 @@
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
                   <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000001080000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln w="9525">
+              <a:miter lim="800000"/>
+              <a:headEnd/>
+              <a:tailEnd/>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="32004" rIns="27432" bIns="32004" anchor="ctr" upright="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr algn="ctr" rtl="0">
+                <a:defRPr sz="1000"/>
+              </a:pPr>
+              <a:r>
+                <a:rPr lang="ko-KR" altLang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike" baseline="0">
+                  <a:solidFill>
+                    <a:srgbClr val="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="맑은 고딕"/>
+                  <a:ea typeface="맑은 고딕"/>
+                </a:rPr>
+                <a:t>"." 값 제거 매크로</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+        <xdr:clientData fPrintsWithSheet="0"/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>18</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>0</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>19</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>2</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="3073" name="Button 1" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s3073"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{821F4EF6-FE8A-4EDC-BFB9-69CCBC42BE37}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2592,4 +2897,882 @@
     </mc:Choice>
   </mc:AlternateContent>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{860628AA-5B4E-4553-A417-B519996C09AB}">
+  <dimension ref="A3:AL217"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
+  <cols>
+    <col min="1" max="1" width="24.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="24.75" customWidth="1"/>
+    <col min="4" max="4" width="255.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="13.125" customWidth="1"/>
+    <col min="10" max="10" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="12.375" customWidth="1"/>
+    <col min="13" max="13" width="12.875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.375" customWidth="1"/>
+    <col min="17" max="17" width="18.75" style="10" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.25" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.375" customWidth="1"/>
+    <col min="24" max="24" width="12" bestFit="1" customWidth="1"/>
+    <col min="25" max="34" width="13.375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:38" ht="17.25" customHeight="1">
+      <c r="A3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3"/>
+      <c r="AA3" s="3"/>
+      <c r="AB3" s="3"/>
+      <c r="AC3" s="3"/>
+      <c r="AD3" s="3"/>
+      <c r="AE3" s="3"/>
+      <c r="AF3" s="3"/>
+      <c r="AG3" s="3"/>
+      <c r="AH3" s="3"/>
+      <c r="AI3" s="3"/>
+      <c r="AJ3" s="3"/>
+      <c r="AK3" s="3"/>
+      <c r="AL3" s="3"/>
+    </row>
+    <row r="4" spans="1:38" ht="17.25" customHeight="1">
+      <c r="A4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="8"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
+      <c r="AA4" s="3"/>
+    </row>
+    <row r="5" spans="1:38">
+      <c r="A5" s="12" t="str">
+        <f>B5&amp;"_"&amp;C5</f>
+        <v>MiniVillagerWoman_Sun2</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="V5" s="6"/>
+    </row>
+    <row r="6" spans="1:38">
+      <c r="A6" s="12" t="str">
+        <f t="shared" ref="A6:A20" si="0">B6&amp;"_"&amp;C6</f>
+        <v>MiniVillagerWoman_Sun_old</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="V6" s="6"/>
+    </row>
+    <row r="7" spans="1:38">
+      <c r="A7" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>MiniVillagerWoman_Sun_17</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="R7" s="6"/>
+      <c r="V7" s="6"/>
+    </row>
+    <row r="8" spans="1:38">
+      <c r="A8" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>MiniVillagerWoman_Sun_18</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="R8" s="6"/>
+      <c r="V8" s="6"/>
+    </row>
+    <row r="9" spans="1:38">
+      <c r="A9" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>MiniVillagerWoman_Sun_nothing</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
+      <c r="R9" s="6"/>
+      <c r="V9" s="6"/>
+    </row>
+    <row r="10" spans="1:38">
+      <c r="A10" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>MiniVillagerWoman_eventSeen_35_memory_oneweek</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="R10" s="6"/>
+      <c r="V10" s="6"/>
+    </row>
+    <row r="11" spans="1:38">
+      <c r="A11" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>MiniVillagerWoman_4</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11">
+        <v>4</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="R11" s="6"/>
+      <c r="V11" s="6"/>
+    </row>
+    <row r="12" spans="1:38">
+      <c r="A12" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>MiniVillagerWoman_Mon</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="R12" s="6"/>
+      <c r="V12" s="6"/>
+    </row>
+    <row r="13" spans="1:38">
+      <c r="A13" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>MiniVillagerWoman_Tue</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" t="s">
+        <v>53</v>
+      </c>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="R13" s="6"/>
+      <c r="V13" s="6"/>
+    </row>
+    <row r="14" spans="1:38">
+      <c r="A14" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>MiniVillagerWoman_Wed</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" t="s">
+        <v>54</v>
+      </c>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="R14" s="6"/>
+    </row>
+    <row r="15" spans="1:38">
+      <c r="A15" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>MiniVillagerWoman_Thu</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" t="s">
+        <v>55</v>
+      </c>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="R15" s="6"/>
+    </row>
+    <row r="16" spans="1:38">
+      <c r="A16" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>MiniVillagerWoman_Fri</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" t="s">
+        <v>56</v>
+      </c>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
+      <c r="R16" s="6"/>
+    </row>
+    <row r="17" spans="1:18">
+      <c r="A17" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>MiniVillagerWoman_Sat</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" t="s">
+        <v>57</v>
+      </c>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="R17" s="6"/>
+    </row>
+    <row r="18" spans="1:18">
+      <c r="A18" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>MiniVillagerWoman_Sun</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" t="s">
+        <v>58</v>
+      </c>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="6"/>
+      <c r="R18" s="6"/>
+    </row>
+    <row r="19" spans="1:18">
+      <c r="A19" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>MiniVillagerWoman_summer_Mon</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" t="s">
+        <v>59</v>
+      </c>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="R19" s="6"/>
+    </row>
+    <row r="20" spans="1:18">
+      <c r="A20" s="12" t="str">
+        <f t="shared" si="0"/>
+        <v>MiniVillagerWoman_summer_Tue</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" t="s">
+        <v>60</v>
+      </c>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
+      <c r="R20" s="6"/>
+    </row>
+    <row r="21" spans="1:18">
+      <c r="A21" s="12" t="str">
+        <f>B21&amp;"_"&amp;C21</f>
+        <v>MiniVillagerWoman_spring_6</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" t="s">
+        <v>61</v>
+      </c>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+      <c r="R21" s="6"/>
+    </row>
+    <row r="22" spans="1:18">
+      <c r="A22" s="12" t="str">
+        <f t="shared" ref="A22:A24" si="1">B22&amp;"_"&amp;C22</f>
+        <v>MiniVillagerWoman_spring_6old</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" t="s">
+        <v>62</v>
+      </c>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+      <c r="R22" s="6"/>
+    </row>
+    <row r="23" spans="1:18">
+      <c r="A23" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>MiniVillagerWoman_spring_61</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C23" t="s">
+        <v>41</v>
+      </c>
+      <c r="D23" t="s">
+        <v>63</v>
+      </c>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="R23" s="6"/>
+    </row>
+    <row r="24" spans="1:18">
+      <c r="A24" s="12" t="str">
+        <f t="shared" si="1"/>
+        <v>MiniVillagerWoman_spring_62</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C24" t="s">
+        <v>42</v>
+      </c>
+      <c r="D24" t="s">
+        <v>64</v>
+      </c>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
+      <c r="R24" s="6"/>
+    </row>
+    <row r="25" spans="1:18">
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
+      <c r="R25" s="6"/>
+    </row>
+    <row r="26" spans="1:18">
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
+      <c r="R26" s="6"/>
+    </row>
+    <row r="27" spans="1:18">
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
+      <c r="R27" s="6"/>
+    </row>
+    <row r="28" spans="1:18">
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="9"/>
+      <c r="R28" s="6"/>
+    </row>
+    <row r="29" spans="1:18">
+      <c r="G29" s="6"/>
+      <c r="H29" s="6"/>
+      <c r="I29" s="6"/>
+      <c r="J29" s="9"/>
+      <c r="R29" s="6"/>
+    </row>
+    <row r="30" spans="1:18">
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+      <c r="I30" s="6"/>
+      <c r="J30" s="9"/>
+      <c r="R30" s="6"/>
+    </row>
+    <row r="31" spans="1:18">
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
+      <c r="J31" s="9"/>
+      <c r="R31" s="6"/>
+    </row>
+    <row r="32" spans="1:18">
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="6"/>
+      <c r="R32" s="6"/>
+    </row>
+    <row r="33" spans="7:18">
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+      <c r="I33" s="6"/>
+      <c r="R33" s="6"/>
+    </row>
+    <row r="34" spans="7:18">
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+      <c r="I34" s="6"/>
+      <c r="J34" s="9"/>
+      <c r="R34" s="6"/>
+    </row>
+    <row r="35" spans="7:18">
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
+      <c r="I35" s="6"/>
+      <c r="J35" s="9"/>
+      <c r="R35" s="6"/>
+    </row>
+    <row r="36" spans="7:18">
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+      <c r="I36" s="6"/>
+      <c r="J36" s="9"/>
+      <c r="R36" s="6"/>
+    </row>
+    <row r="37" spans="7:18">
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="9"/>
+      <c r="R37" s="6"/>
+    </row>
+    <row r="38" spans="7:18">
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
+      <c r="I38" s="6"/>
+      <c r="J38" s="9"/>
+      <c r="R38" s="6"/>
+    </row>
+    <row r="39" spans="7:18">
+      <c r="G39" s="6"/>
+      <c r="H39" s="6"/>
+      <c r="I39" s="6"/>
+      <c r="J39" s="9"/>
+      <c r="R39" s="6"/>
+    </row>
+    <row r="40" spans="7:18">
+      <c r="G40" s="6"/>
+      <c r="H40" s="6"/>
+      <c r="I40" s="6"/>
+      <c r="J40" s="9"/>
+      <c r="R40" s="6"/>
+    </row>
+    <row r="41" spans="7:18">
+      <c r="G41" s="6"/>
+      <c r="H41" s="6"/>
+      <c r="I41" s="6"/>
+      <c r="J41" s="9"/>
+      <c r="R41" s="6"/>
+    </row>
+    <row r="42" spans="7:18">
+      <c r="G42" s="6"/>
+      <c r="H42" s="6"/>
+      <c r="I42" s="6"/>
+      <c r="J42" s="9"/>
+      <c r="R42" s="6"/>
+    </row>
+    <row r="43" spans="7:18">
+      <c r="G43" s="6"/>
+      <c r="H43" s="6"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="9"/>
+      <c r="R43" s="6"/>
+    </row>
+    <row r="44" spans="7:18">
+      <c r="G44" s="6"/>
+      <c r="H44" s="6"/>
+      <c r="I44" s="6"/>
+      <c r="J44" s="9"/>
+      <c r="R44" s="6"/>
+    </row>
+    <row r="150" spans="4:4">
+      <c r="D150" s="5"/>
+    </row>
+    <row r="151" spans="4:4">
+      <c r="D151" s="5"/>
+    </row>
+    <row r="152" spans="4:4">
+      <c r="D152" s="5"/>
+    </row>
+    <row r="153" spans="4:4">
+      <c r="D153" s="5"/>
+    </row>
+    <row r="154" spans="4:4">
+      <c r="D154" s="5"/>
+    </row>
+    <row r="155" spans="4:4">
+      <c r="D155" s="5"/>
+    </row>
+    <row r="156" spans="4:4">
+      <c r="D156" s="5"/>
+    </row>
+    <row r="157" spans="4:4">
+      <c r="D157" s="5"/>
+    </row>
+    <row r="158" spans="4:4">
+      <c r="D158" s="5"/>
+    </row>
+    <row r="159" spans="4:4">
+      <c r="D159" s="5"/>
+    </row>
+    <row r="160" spans="4:4">
+      <c r="D160" s="5"/>
+    </row>
+    <row r="161" spans="4:4">
+      <c r="D161" s="5"/>
+    </row>
+    <row r="162" spans="4:4">
+      <c r="D162" s="5"/>
+    </row>
+    <row r="163" spans="4:4">
+      <c r="D163" s="5"/>
+    </row>
+    <row r="164" spans="4:4">
+      <c r="D164" s="5"/>
+    </row>
+    <row r="165" spans="4:4">
+      <c r="D165" s="5"/>
+    </row>
+    <row r="166" spans="4:4">
+      <c r="D166" s="5"/>
+    </row>
+    <row r="167" spans="4:4">
+      <c r="D167" s="5"/>
+    </row>
+    <row r="168" spans="4:4">
+      <c r="D168" s="5"/>
+    </row>
+    <row r="169" spans="4:4">
+      <c r="D169" s="5"/>
+    </row>
+    <row r="170" spans="4:4">
+      <c r="D170" s="5"/>
+    </row>
+    <row r="171" spans="4:4">
+      <c r="D171" s="5"/>
+    </row>
+    <row r="172" spans="4:4">
+      <c r="D172" s="5"/>
+    </row>
+    <row r="173" spans="4:4">
+      <c r="D173" s="5"/>
+    </row>
+    <row r="174" spans="4:4">
+      <c r="D174" s="5"/>
+    </row>
+    <row r="175" spans="4:4">
+      <c r="D175" s="5"/>
+    </row>
+    <row r="176" spans="4:4">
+      <c r="D176" s="5"/>
+    </row>
+    <row r="177" spans="4:4">
+      <c r="D177" s="5"/>
+    </row>
+    <row r="178" spans="4:4">
+      <c r="D178" s="5"/>
+    </row>
+    <row r="179" spans="4:4">
+      <c r="D179" s="5"/>
+    </row>
+    <row r="180" spans="4:4">
+      <c r="D180" s="5"/>
+    </row>
+    <row r="181" spans="4:4">
+      <c r="D181" s="5"/>
+    </row>
+    <row r="182" spans="4:4">
+      <c r="D182" s="5"/>
+    </row>
+    <row r="183" spans="4:4">
+      <c r="D183" s="5"/>
+    </row>
+    <row r="184" spans="4:4">
+      <c r="D184" s="5"/>
+    </row>
+    <row r="185" spans="4:4">
+      <c r="D185" s="5"/>
+    </row>
+    <row r="186" spans="4:4">
+      <c r="D186" s="5"/>
+    </row>
+    <row r="187" spans="4:4">
+      <c r="D187" s="5"/>
+    </row>
+    <row r="188" spans="4:4">
+      <c r="D188" s="5"/>
+    </row>
+    <row r="189" spans="4:4">
+      <c r="D189" s="5"/>
+    </row>
+    <row r="190" spans="4:4">
+      <c r="D190" s="5"/>
+    </row>
+    <row r="191" spans="4:4">
+      <c r="D191" s="5"/>
+    </row>
+    <row r="192" spans="4:4">
+      <c r="D192" s="5"/>
+    </row>
+    <row r="193" spans="4:4">
+      <c r="D193" s="5"/>
+    </row>
+    <row r="194" spans="4:4">
+      <c r="D194" s="5"/>
+    </row>
+    <row r="195" spans="4:4">
+      <c r="D195" s="5"/>
+    </row>
+    <row r="196" spans="4:4">
+      <c r="D196" s="5"/>
+    </row>
+    <row r="197" spans="4:4">
+      <c r="D197" s="5"/>
+    </row>
+    <row r="198" spans="4:4">
+      <c r="D198" s="5"/>
+    </row>
+    <row r="199" spans="4:4">
+      <c r="D199" s="5"/>
+    </row>
+    <row r="200" spans="4:4">
+      <c r="D200" s="5"/>
+    </row>
+    <row r="201" spans="4:4">
+      <c r="D201" s="5"/>
+    </row>
+    <row r="202" spans="4:4">
+      <c r="D202" s="5"/>
+    </row>
+    <row r="203" spans="4:4">
+      <c r="D203" s="5"/>
+    </row>
+    <row r="204" spans="4:4">
+      <c r="D204" s="5"/>
+    </row>
+    <row r="205" spans="4:4">
+      <c r="D205" s="5"/>
+    </row>
+    <row r="206" spans="4:4">
+      <c r="D206" s="5"/>
+    </row>
+    <row r="207" spans="4:4">
+      <c r="D207" s="5"/>
+    </row>
+    <row r="208" spans="4:4">
+      <c r="D208" s="5"/>
+    </row>
+    <row r="209" spans="4:4">
+      <c r="D209" s="5"/>
+    </row>
+    <row r="210" spans="4:4">
+      <c r="D210" s="5"/>
+    </row>
+    <row r="211" spans="4:4">
+      <c r="D211" s="5"/>
+    </row>
+    <row r="212" spans="4:4">
+      <c r="D212" s="5"/>
+    </row>
+    <row r="213" spans="4:4">
+      <c r="D213" s="5"/>
+    </row>
+    <row r="214" spans="4:4">
+      <c r="D214" s="5"/>
+    </row>
+    <row r="215" spans="4:4">
+      <c r="D215" s="5"/>
+    </row>
+    <row r="216" spans="4:4">
+      <c r="D216" s="5"/>
+    </row>
+    <row r="217" spans="4:4">
+      <c r="D217" s="5"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x14">
+      <controls>
+        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+          <mc:Choice Requires="x14">
+            <control shapeId="3073" r:id="rId4" name="Button 1">
+              <controlPr defaultSize="0" print="0" autoFill="0" autoPict="0" macro="[0]!DeleteSpecificValueCells">
+                <anchor moveWithCells="1" sizeWithCells="1">
+                  <from>
+                    <xdr:col>18</xdr:col>
+                    <xdr:colOff>0</xdr:colOff>
+                    <xdr:row>0</xdr:row>
+                    <xdr:rowOff>0</xdr:rowOff>
+                  </from>
+                  <to>
+                    <xdr:col>19</xdr:col>
+                    <xdr:colOff>0</xdr:colOff>
+                    <xdr:row>2</xdr:row>
+                    <xdr:rowOff>0</xdr:rowOff>
+                  </to>
+                </anchor>
+              </controlPr>
+            </control>
+          </mc:Choice>
+        </mc:AlternateContent>
+      </controls>
+    </mc:Choice>
+  </mc:AlternateContent>
+</worksheet>
 </file>
</xml_diff>